<commit_message>
Cement review: demand/trade restructure, phase A costs and CCS, regional input rows
- BCD now apparent consumption grown on AEO cement-and-lime index; BCtCR is the blend ratio
- New BFoCDMbNI net-import share and Domestic Clinker Demand; MACtCR replaces PACS and MASCM
- Kiln fuel mix trended in-model from BIFU 239; CNBEIR unit fix; smoothed utilization for investment decisions
- Capital costs moved to 2012 USD; CRSW recalibrated (0.0357 to 0.1297)
- Cement CCS reconciled with the CCS sector (capture capital, operating cost, sequestered tons to 239)
- Petcoke and fossil alternative-fuel emission corrections
- Region drop-down on all cement input workbooks; non-US rows loaded from research drafts (US CSVs unchanged)
</commit_message>
<xml_diff>
--- a/InputData/indst/CEIbPaF/Cement Energy Intensity by Pathway and Fuel.xlsx
+++ b/InputData/indst/CEIbPaF/Cement Energy Intensity by Pathway and Fuel.xlsx
@@ -1007,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1087,6 +1087,34 @@
         <is>
           <t>EI internal engineering estimate; no company disclosure</t>
         </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Petcoke split between EPS fuel elements, following BIFU: AEO cement block 2025 petroleum coke 24.6 TBtu (filed as petroleum diesel) vs other petroleum 35.4 TBtu (filed as residual-oil feedstock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Share of module petcoke on petroleum diesel</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Share on heavy or residual fuel oil</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>1-B10</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1180,11 +1208,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>heavy or residual fuel oil if (petroleum coke)</t>
+          <t>heavy or residual fuel oil if (petroleum coke, 59%)</t>
         </is>
       </c>
       <c r="B9">
-        <f>ROUND($B$2*Parameters!$B$3,-4)</f>
+        <f>ROUND($B$2*Parameters!$B$3*Parameters!$B$11,-3)</f>
         <v/>
       </c>
     </row>
@@ -1199,6 +1227,17 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>petroleum diesel if (petroleum coke, 41%)</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>ROUND($B$2*Parameters!$B$3*Parameters!$B$10,-3)</f>
+        <v/>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -1242,7 +1281,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Dry kiln with CCS (base + amine adders)</t>
+          <t>CCS pathway: KILN ONLY since 2026-10-01 (capture energy comes from the CCS sector's CC Energy Use per Ton Industry CO2 Sequestered x captured tons); rows equal the dry kiln</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1498,7 @@
         <v/>
       </c>
       <c r="D9">
-        <f>Calc!B18</f>
+        <f>Calc!B15</f>
         <v/>
       </c>
       <c r="E9">
@@ -1507,7 +1546,7 @@
         <v/>
       </c>
       <c r="D11">
-        <f>Calc!B19</f>
+        <f>Calc!B8</f>
         <v/>
       </c>
       <c r="E11">
@@ -1651,7 +1690,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Unit: BTU/metric ton clinker (DRAFT: DOE Bandwidth 2017 thermal x PCA 2023 fuel mix; coal 33%/NG 31%/petcoke-&gt;resid 20%/alt fuels-&gt;biomass 16%; CCS adds amine energy; electric kiln/alt chem placeholders - verify before release)</t>
+          <t>Unit: BTU/metric ton clinker (DOE Bandwidth 2017 thermal x PCA 2023 fuel mix; coal 33%/NG 31%/petcoke 20%/alt fuels 16% (as biomass); petcoke split 41% petroleum diesel + 59% residual oil to mirror BIFU's labelling of AEO petroleum coke and other petroleum (2026-10-01); CCS row is KILN ONLY - capture energy is booked by the CCS sector from captured tons; electric kiln/alt chem placeholders - verify before release)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -1734,7 +1773,7 @@
         <v>550000</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>283000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1743,7 +1782,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>690000</v>
+        <v>407000</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -1765,19 +1804,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>740000</v>
+        <v>590000</v>
       </c>
       <c r="C3" t="n">
         <v>1130000</v>
       </c>
       <c r="D3" t="n">
-        <v>3160000</v>
+        <v>1060000</v>
       </c>
       <c r="E3" t="n">
         <v>550000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>283000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1786,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>690000</v>
+        <v>407000</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>

</xml_diff>